<commit_message>
NR-01: HSE Indicator Tool de volta como referência internacional complementar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NR01/Mapa_item_a_item_das_fontes.xlsx
+++ b/NR01/Mapa_item_a_item_das_fontes.xlsx
@@ -16,12 +16,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hierarquia das fontes" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mapa por item'!$A$3:$K$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mapa por item'!$A$3:$L$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cobertura por fator'!$A$3:$G$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Itens dos originais sem par'!$A$3:$E$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Fontes e licenças'!$A$3:$K$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Fontes e licenças'!$A$3:$K$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Base legal'!$A$3:$E$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Hierarquia das fontes'!$A$3:$D$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Hierarquia das fontes'!$A$3:$D$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -581,152 +581,152 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Complementares, também validados no Brasil: Job Stress Scale (USP, 2004), ERI versão brasileira (Fiocruz, 2008) e PROART (UnB, 2013).O questionário também não é obrigatório (Manual do GRO, 2026, item 17.1.1); se usado, deve ter validação científica, anonimato e participação.</t>
+          <t>Complementares, também validados no Brasil: Job Stress Scale (USP, 2004), ERI versão brasileira (Fiocruz, 2008) e PROART (UnB, 2013).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Referência internacional complementar: HSE Indicator Tool (Health and Safety Executive, Reino Unido), seis fatores de estresse: demandas, controle, suporte, relacionamentos, papel e mudanças.O questionário também não é obrigatório (Manual do GRO, 2026, item 17.1.1); se usado, deve ter validação científica, anonimato e participação.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>A NR-01 e o guia do MTE não indicam nem aprovam questionário. O guia pede fundamentação científica, adequação ao risco e anonimato.</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Este mapa documenta a fundamentação: cada item P&amp;C aponta a fonte oficial e, quando existe, o instrumento validado que o sustenta.</t>
+          <t>A NR-01 e o guia do MTE não indicam nem aprovam questionário. O guia pede fundamentação científica, adequação ao risco e anonimato.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>Este mapa documenta a fundamentação: cada item P&amp;C aponta a fonte oficial e, quando existe, o instrumento validado que o sustenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Os itens P&amp;C são redação própria. Não copiar itens do ERI em produto comercial sem autorização do titular.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Sobre as datas dos originais</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>O ano de cada instrumento é o ano da versão validada, não sinal de desatualização. Questionário validado não é revisto todo ano:</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>mudar as perguntas invalida a validação. O que precisa estar atualizado é a base legal (aba Base legal), e ela está vigente.</t>
+          <t>O ano de cada instrumento é o ano da versão validada, não sinal de desatualização. Questionário validado não é revisto todo ano:</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>mudar as perguntas invalida a validação. O que precisa estar atualizado é a base legal (aba Base legal), e ela está vigente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>Vigente: versão atual confirmada na fonte oficial. Vigente (conferir): em uso, mas sem confirmação de que nada mudou.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Abas</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Mapa por item: cada afirmação P&amp;C com o item original que a sustenta.</t>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Pastas de fontes</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Cobertura por fator: quanto de cada fator do guia tem base em instrumento validado.</t>
+          <t>1. Fontes oficiais MTE: normas e publicações do Ministério do Trabalho.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Itens dos originais sem par: o que os originais perguntam e nós não, com sugestão de incluir ou não.</t>
+          <t>2. Questionarios validados no Brasil: artigos, teses e documentos de validação.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Fontes e licenças: versão, situação, validação no Brasil, licença e como citar cada original.</t>
+          <t>3. Questionarios oficiais usados como base: só os formulários oficiais de cada questionário (COPSOQ II-Br, Job Stress Scale, ERI, PROART e HSE), prontos para apresentar.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Base legal: normas que fundamentam o kit e sua situação.</t>
-        </is>
-      </c>
+      <c r="A26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Hierarquia das fontes: oficial brasileira e científica validada no Brasil.</t>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Abas</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Mapa por item: cada afirmação P&amp;C com o item original que a sustenta.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>Texto sugerido para documento ao cliente</t>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Cobertura por fator: quanto de cada fator do guia tem base em instrumento validado.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>O questionário foi elaborado pela Peixoto &amp; Cury a partir dos 13 fatores do Guia de informações sobre os fatores de riscos psicossociais</t>
+          <t>Itens dos originais sem par: o que os originais perguntam e nós não, com sugestão de incluir ou não.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>relacionados ao trabalho (MTE) e do Manual do GRO (MTE, 2026), em atendimento ao subitem 1.5.3.1.4 da NR-01, com fundamentação em</t>
+          <t>Fontes e licenças: versão, situação, validação no Brasil, licença e como citar cada original.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>questionário validado no Brasil COPSOQ II-Br (Gonçalves et al., 2021; Sato et al., Fundacentro, 2026), complementado pela Job Stress Scale,</t>
+          <t>Base legal: normas que fundamentam o kit e sua situação.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>pelo ERI e pelo PROART, e na legislação trabalhista (CLT e Lei nº 14.457/2022).</t>
+          <t>Hierarquia das fontes: oficial brasileira e científica validada no Brasil.</t>
         </is>
       </c>
     </row>
@@ -734,7 +734,45 @@
       <c r="A34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Texto sugerido para documento ao cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>O questionário foi elaborado pela Peixoto &amp; Cury a partir dos 13 fatores do Guia de informações sobre os fatores de riscos psicossociais</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>relacionados ao trabalho (MTE) e do Manual do GRO (MTE, 2026), em atendimento ao subitem 1.5.3.1.4 da NR-01, com fundamentação em</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>questionário validado no Brasil COPSOQ II-Br (Gonçalves et al., 2021; Sato et al., Fundacentro, 2026), complementado pela Job Stress Scale,</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>pelo ERI e pelo PROART, com o HSE Indicator Tool (Reino Unido) como referência internacional, e na legislação trabalhista (CLT e Lei nº 14.457/2022).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Consulta às fontes em 20/10/2026. O mapeamento item a item foi feito por comparação de texto; recomenda-se revisão por profissional de SST.</t>
         </is>
@@ -751,7 +789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -764,7 +802,8 @@
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="34" customWidth="1" min="9" max="9"/>
     <col width="38" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -827,6 +866,11 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
+          <t>HSE Indicator Tool (referência internacional, Reino Unido)</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
           <t>Observação</t>
         </is>
       </c>
@@ -884,6 +928,12 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
+          <t>HSE 6 (Demandas): I have unachievable deadlines
+HSE 22 (Demandas): I have unrealistic time pressures</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
           <t>Mesmo conceito do DCSQ d; acrescentamos "com qualidade".</t>
         </is>
       </c>
@@ -937,7 +987,13 @@
           <t>EOPT12 (Organização prescrita do trabalho): O ritmo de trabalho é adequado</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr"/>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>HSE 9 (Demandas): I have to work very intensively
+HSE 20 (Demandas): I have to work very fast</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -992,6 +1048,11 @@
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>HSE 12 (Demandas): I have to neglect some tasks because I have too much to do</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>Originais medem excesso de trabalho; nós amarramos o volume à jornada.</t>
         </is>
@@ -1036,7 +1097,12 @@
       <c r="H7" s="5" t="inlineStr"/>
       <c r="I7" s="5" t="inlineStr"/>
       <c r="J7" s="5" t="inlineStr"/>
-      <c r="K7" s="5" t="inlineStr"/>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>HSE 18 (Demandas): I am pressured to work long hours</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1079,6 +1145,7 @@
       <c r="I8" s="5" t="inlineStr"/>
       <c r="J8" s="5" t="inlineStr"/>
       <c r="K8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1117,6 +1184,12 @@
       <c r="J9" s="5" t="inlineStr"/>
       <c r="K9" s="5" t="inlineStr">
         <is>
+          <t>HSE 2 (Controle): I can decide when to take a break
+HSE 16 (Demandas): I am unable to take sufficient breaks</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
           <t>Item próprio: pausas e intervalo, base na CLT.</t>
         </is>
       </c>
@@ -1168,6 +1241,12 @@
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
+          <t>HSE 6 (Demandas): I have unachievable deadlines
+HSE 22 (Demandas): I have unrealistic time pressures</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
           <t>PROART mede flexibilidade de prazos e condições para atingir resultados.</t>
         </is>
       </c>
@@ -1220,7 +1299,8 @@
 ESPT9 (Sofrimento patogênico no trabalho): Minhas tarefas são banais</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr"/>
+      <c r="L11" s="5" t="inlineStr">
         <is>
           <t>PROART capta o efeito (improdutividade, tarefas banais); nenhum original pergunta diretamente sobre ociosidade.</t>
         </is>
@@ -1275,7 +1355,8 @@
           <t>EOPT17 (Organização prescrita do trabalho): As tarefas que executo em meu trabalho são variadas</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="inlineStr">
         <is>
           <t>DCSQ mede uso de habilidades (dimensão controle).</t>
         </is>
@@ -1328,7 +1409,14 @@
           <t>EOPT9 (Organização prescrita do trabalho): Tenho autonomia para realizar as tarefas como julgo melhor</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr"/>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>HSE 15 (Controle): I have a choice in deciding how I do my work
+HSE 10 (Controle): I have a say in my own work speed
+HSE 25 (Controle): I have some say over the way I work</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1378,6 +1466,11 @@
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>HSE 19 (Controle): I have a choice in deciding what I do at work</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
         <is>
           <t>Originais falam em decidir o que fazer; nós falamos em distribuição de tarefas na equipe.</t>
         </is>
@@ -1426,7 +1519,12 @@
           <t>EOPT18 (Organização prescrita do trabalho): Tenho liberdade para opinar sobre o meu trabalho</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr"/>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>HSE 25 (Controle): I have some say over the way I work</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1478,6 +1576,12 @@
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
+          <t>HSE 23 (Apoio da chefia): I can rely on my line manager to help me out with a work problem
+HSE 29 (Apoio da chefia): I can talk to my line manager about something that has upset or annoyed me about work</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
           <t>DCSQ mede relação com a chefia; PROART, liberdade para dialogar com ela.</t>
         </is>
       </c>
@@ -1521,7 +1625,13 @@
       </c>
       <c r="I17" s="5" t="inlineStr"/>
       <c r="J17" s="5" t="inlineStr"/>
-      <c r="K17" s="5" t="inlineStr"/>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>HSE 7 (Apoio dos colegas): If work gets difficult, my colleagues will help me
+HSE 24 (Apoio dos colegas): I get help and support I need from colleagues</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1568,6 +1678,11 @@
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
+          <t>HSE 8 (Apoio da chefia): I am given supportive feedback on the work I do</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
           <t>PROART mede indiferença da chefia com o trabalho.</t>
         </is>
       </c>
@@ -1616,6 +1731,7 @@
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr"/>
+      <c r="L19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1661,7 +1777,13 @@
           <t>ESPT25 (Sofrimento patogênico no trabalho): É difícil a convivência com meus colegas</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr"/>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>HSE 34 (Relacionamentos): Relationships at work are strained
+HSE 14 (Relacionamentos): There is friction or anger between colleagues</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1702,7 +1824,12 @@
       <c r="H21" s="5" t="inlineStr"/>
       <c r="I21" s="5" t="inlineStr"/>
       <c r="J21" s="5" t="inlineStr"/>
-      <c r="K21" s="5" t="inlineStr"/>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>HSE 14 (Relacionamentos): There is friction or anger between colleagues</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1747,7 +1874,12 @@
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr"/>
-      <c r="K22" s="5" t="inlineStr"/>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>HSE 27 (Apoio dos colegas): I receive the respect at work I deserve from my colleagues</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1793,7 +1925,13 @@
 EOPT11 (Organização prescrita do trabalho): As informações de que preciso para executar minhas tarefas são claras</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr"/>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>HSE 1 (Papel): I am clear what is expected of me at work
+HSE 4 (Papel): I know how to go about getting my job done</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1839,7 +1977,12 @@
           <t>EOPT5 (Organização prescrita do trabalho): Há clareza na definição das tarefas</t>
         </is>
       </c>
-      <c r="K24" s="5" t="inlineStr"/>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>HSE 11 (Papel): I am clear what my duties and responsibilities are</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1884,7 +2027,12 @@
           <t>EOPT16 (Organização prescrita do trabalho): As orientações que me são passadas para realizar as tarefas são coerentes entre si</t>
         </is>
       </c>
-      <c r="K25" s="5" t="inlineStr"/>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>HSE 3 (Demandas): Different groups at work demand things from me that are hard to combine</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1935,6 +2083,7 @@
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr"/>
+      <c r="L26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1980,6 +2129,7 @@
       <c r="I27" s="5" t="inlineStr"/>
       <c r="J27" s="5" t="inlineStr"/>
       <c r="K27" s="5" t="inlineStr"/>
+      <c r="L27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -2026,6 +2176,7 @@
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr"/>
+      <c r="L28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -2068,6 +2219,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr"/>
       <c r="K29" s="5" t="inlineStr"/>
+      <c r="L29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -2112,7 +2264,8 @@
           <t>EOPT6 (Organização prescrita do trabalho): Há justiça na distribuição das tarefas</t>
         </is>
       </c>
-      <c r="K30" s="5" t="inlineStr">
+      <c r="K30" s="5" t="inlineStr"/>
+      <c r="L30" s="5" t="inlineStr">
         <is>
           <t>PROART cobre só distribuição de tarefas. DCSQ e ERI não medem justiça.</t>
         </is>
@@ -2163,6 +2316,7 @@
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr"/>
+      <c r="L31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -2204,6 +2358,7 @@
       <c r="I32" s="5" t="inlineStr"/>
       <c r="J32" s="5" t="inlineStr"/>
       <c r="K32" s="5" t="inlineStr"/>
+      <c r="L32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -2249,6 +2404,11 @@
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>HSE 32 (Mudanças): When changes are made at work, I am clear how they will work out in practice</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
         <is>
           <t>PROART mede se o ambiente se desorganiza com mudanças; nós medimos antecedência da informação.</t>
         </is>
@@ -2289,7 +2449,8 @@
       <c r="H34" s="5" t="inlineStr"/>
       <c r="I34" s="5" t="inlineStr"/>
       <c r="J34" s="5" t="inlineStr"/>
-      <c r="K34" s="5" t="inlineStr">
+      <c r="K34" s="5" t="inlineStr"/>
+      <c r="L34" s="5" t="inlineStr">
         <is>
           <t>Item próprio (treinamento em sistemas novos).</t>
         </is>
@@ -2340,6 +2501,12 @@
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
+          <t>HSE 28 (Mudanças): Staff are always consulted about change at work
+HSE 26 (Mudanças): I have sufficient opportunities to question managers about change at work</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
           <t>PROART mede participação nas decisões sobre o trabalho.</t>
         </is>
       </c>
@@ -2383,7 +2550,13 @@
       <c r="H36" s="5" t="inlineStr"/>
       <c r="I36" s="5" t="inlineStr"/>
       <c r="J36" s="5" t="inlineStr"/>
-      <c r="K36" s="5" t="inlineStr"/>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>HSE 5 (Relacionamentos): I am subject to personal harassment in the form of unkind words or behaviour
+HSE 21 (Relacionamentos): I am subject to bullying at work</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -2420,7 +2593,8 @@
       <c r="H37" s="5" t="inlineStr"/>
       <c r="I37" s="5" t="inlineStr"/>
       <c r="J37" s="5" t="inlineStr"/>
-      <c r="K37" s="5" t="inlineStr">
+      <c r="K37" s="5" t="inlineStr"/>
+      <c r="L37" s="5" t="inlineStr">
         <is>
           <t>Item próprio: testemunha de assédio, base na Lei 14.457/2022.</t>
         </is>
@@ -2465,7 +2639,12 @@
       <c r="H38" s="5" t="inlineStr"/>
       <c r="I38" s="5" t="inlineStr"/>
       <c r="J38" s="5" t="inlineStr"/>
-      <c r="K38" s="5" t="inlineStr"/>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>HSE 5 (Relacionamentos): I am subject to personal harassment in the form of unkind words or behaviour</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -2502,7 +2681,8 @@
       <c r="H39" s="5" t="inlineStr"/>
       <c r="I39" s="5" t="inlineStr"/>
       <c r="J39" s="5" t="inlineStr"/>
-      <c r="K39" s="5" t="inlineStr">
+      <c r="K39" s="5" t="inlineStr"/>
+      <c r="L39" s="5" t="inlineStr">
         <is>
           <t>Item próprio sobre canal de denúncia (Lei 14.457/2022 e NR-05).</t>
         </is>
@@ -2548,6 +2728,7 @@
       <c r="I40" s="5" t="inlineStr"/>
       <c r="J40" s="5" t="inlineStr"/>
       <c r="K40" s="5" t="inlineStr"/>
+      <c r="L40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -2589,7 +2770,8 @@
       <c r="H41" s="5" t="inlineStr"/>
       <c r="I41" s="5" t="inlineStr"/>
       <c r="J41" s="5" t="inlineStr"/>
-      <c r="K41" s="5" t="inlineStr">
+      <c r="K41" s="5" t="inlineStr"/>
+      <c r="L41" s="5" t="inlineStr">
         <is>
           <t>Idem.</t>
         </is>
@@ -2632,6 +2814,11 @@
       <c r="J42" s="5" t="inlineStr"/>
       <c r="K42" s="5" t="inlineStr">
         <is>
+          <t>HSE 33 (Apoio da chefia): I am supported through emotionally demanding work</t>
+        </is>
+      </c>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
           <t>Item próprio: apoio após evento grave.</t>
         </is>
       </c>
@@ -2680,6 +2867,7 @@
         </is>
       </c>
       <c r="K43" s="5" t="inlineStr"/>
+      <c r="L43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -2722,6 +2910,7 @@
         </is>
       </c>
       <c r="K44" s="5" t="inlineStr"/>
+      <c r="L44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -2769,6 +2958,7 @@
         </is>
       </c>
       <c r="K45" s="5" t="inlineStr"/>
+      <c r="L45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -2805,7 +2995,8 @@
       <c r="H46" s="5" t="inlineStr"/>
       <c r="I46" s="5" t="inlineStr"/>
       <c r="J46" s="5" t="inlineStr"/>
-      <c r="K46" s="5" t="inlineStr">
+      <c r="K46" s="5" t="inlineStr"/>
+      <c r="L46" s="5" t="inlineStr">
         <is>
           <t>Item próprio: fator do guia do MTE sem correspondente nos questionários validados.</t>
         </is>
@@ -2851,7 +3042,8 @@
 EOPT4 (Organização prescrita do trabalho): Os equipamentos são adequados para a realização das tarefas</t>
         </is>
       </c>
-      <c r="K47" s="5" t="inlineStr">
+      <c r="K47" s="5" t="inlineStr"/>
+      <c r="L47" s="5" t="inlineStr">
         <is>
           <t>PROART mede recursos e equipamentos em geral, sem recorte de trabalho remoto.</t>
         </is>
@@ -2892,14 +3084,15 @@
       <c r="H48" s="5" t="inlineStr"/>
       <c r="I48" s="5" t="inlineStr"/>
       <c r="J48" s="5" t="inlineStr"/>
-      <c r="K48" s="5" t="inlineStr">
+      <c r="K48" s="5" t="inlineStr"/>
+      <c r="L48" s="5" t="inlineStr">
         <is>
           <t>Item próprio: fator do guia do MTE sem correspondente nos questionários validados.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:K48"/>
+  <autoFilter ref="A3:L48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3978,7 +4171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4391,7 +4584,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>(a baixar) Gonçalves et al 2021</t>
+          <t>2. Questionarios validados no Brasil/COPSOQ II-Br - validacao Goncalves et al 2021 Rev Saude Publica USP.pdf</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -4441,39 +4634,39 @@
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>Download bloqueado pelo site neste ambiente; baixar pelo navegador. DOI 10.11606/s1518-8787.2021055003123. Questionário completo na tese de Gonçalves (UFSCar, 2019).</t>
+          <t>DOI 10.11606/s1518-8787.2021055003123. Formulário oficial em 3. Questionarios oficiais usados como base.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>2. Questionarios validados no Brasil/ERI - questionario versao brasileira curta.pdf</t>
+          <t>2. Questionarios validados no Brasil/COPSOQ II-Br - tese UFSCar Goncalves 2019 (completa).pdf</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Effort-Reward Imbalance (ERI), versão curta</t>
+          <t>Tese de doutorado com o processo de validação</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Instituto de Sociologia Médica, Univ. Düsseldorf (Siegrist)</t>
+          <t>Universidade Federal de São Carlos (UFSCar), Programa de Pós-Graduação em Fisioterapia</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>uniklinik-duesseldorf.de (página "ERI questionnaires")</t>
+          <t>repositorio.ufscar.br/handle/ufscar/11763</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Validação brasileira de 2008</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Arquivo distribuído hoje no site oficial do instituto; as perguntas são as da validação brasileira de 2008.</t>
+          <t>Ano da tese que originou a validação publicada em 2021.</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -4483,44 +4676,44 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Sim: Chor et al., 2008 (alfa de Cronbach 0,68 esforço; 0,78 recompensa; 0,78 comprometimento excessivo).</t>
+          <t>Sim: origem da versão brasileira.</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Livre só para pesquisa e ensino. Uso comercial exige autorização do Prof. Johannes Siegrist.</t>
+          <t>Acesso aberto; citar a fonte.</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>CHOR, D. et al. The Brazilian version of the effort-reward imbalance questionnaire to assess job stress. Cadernos de Saúde Pública, Rio de Janeiro, v. 24, n. 1, p. 219-224, 2008.</t>
+          <t>GONÇALVES, J. S. Os aspectos psicossociais no trabalho. 2019. Tese (Doutorado em Fisioterapia) - Universidade Federal de São Carlos, São Carlos, 2019.</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>Versão brasileira coordenada por Rosane Härter Griep. Por causa da licença, a P&amp;C não reproduz os itens: usa redação própria e cita o modelo.</t>
+          <t>Formulário final no Apêndice VIII (p. 78 a 81), extraído para a pasta 3.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2. Questionarios validados no Brasil/ERI - questionario versao brasileira longa.pdf</t>
+          <t>2. Questionarios validados no Brasil/ERI - questionario versao brasileira curta.pdf</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Effort-Reward Imbalance (ERI), versão longa</t>
+          <t>Effort-Reward Imbalance (ERI), versão curta</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Idem</t>
+          <t>Instituto de Sociologia Médica, Univ. Düsseldorf (Siegrist)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Idem</t>
+          <t>uniklinik-duesseldorf.de (página "ERI questionnaires")</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -4530,7 +4723,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Idem.</t>
+          <t>Arquivo distribuído hoje no site oficial do instituto; as perguntas são as da validação brasileira de 2008.</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -4540,50 +4733,54 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Idem.</t>
+          <t>Sim: Chor et al., 2008 (alfa de Cronbach 0,68 esforço; 0,78 recompensa; 0,78 comprometimento excessivo).</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Idem.</t>
+          <t>Livre só para pesquisa e ensino. Uso comercial exige autorização do Prof. Johannes Siegrist.</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Idem.</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr"/>
+          <t>CHOR, D. et al. The Brazilian version of the effort-reward imbalance questionnaire to assess job stress. Cadernos de Saúde Pública, Rio de Janeiro, v. 24, n. 1, p. 219-224, 2008.</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Versão brasileira coordenada por Rosane Härter Griep. Por causa da licença, a P&amp;C não reproduz os itens: usa redação própria e cita o modelo.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>2. Questionarios validados no Brasil/Job Stress Scale (DCSQ) - validacao brasileira Alves et al 2004.pdf</t>
+          <t>2. Questionarios validados no Brasil/ERI - questionario versao brasileira longa.pdf</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Job Stress Scale / DCSQ (modelo demanda-controle de Karasek, versão sueca de Theorell)</t>
+          <t>Effort-Reward Imbalance (ERI), versão longa</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Revista de Saúde Pública (USP), v. 38, n. 2, p. 164-171</t>
+          <t>Idem</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>scielo.br/j/rsp/a/55vCVJNvKpJcsGNjhpq5W4r</t>
+          <t>Idem</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>2004 (17 itens)</t>
+          <t>Validação brasileira de 2008</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Ano da adaptação e validação para o português.</t>
+          <t>Idem.</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -4593,133 +4790,349 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Sim: o próprio artigo (reprodutibilidade 0,88 demanda; 0,87 controle; 0,85 apoio social).</t>
+          <t>Idem.</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Artigo de acesso aberto; itens no anexo. O JCQ original de Karasek (versão longa) é licenciado e não foi usado.</t>
+          <t>Idem.</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>ALVES, M. G. M. et al. Versão resumida da "job stress scale": adaptação para o português. Revista de Saúde Pública, São Paulo, v. 38, n. 2, p. 164-171, 2004.</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>Continua sendo a versão de referência no Brasil. DOI 10.1590/S0034-89102004000200003.</t>
-        </is>
-      </c>
+          <t>Idem.</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2. Questionarios validados no Brasil/PROART - tese UnB Facas 2013 (protocolo no Anexo 5).pdf</t>
+          <t>2. Questionarios validados no Brasil/Job Stress Scale (DCSQ) - validacao brasileira Alves et al 2004.pdf</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Protocolo de Avaliação dos Riscos Psicossociais no Trabalho (PROART)</t>
+          <t>Job Stress Scale / DCSQ (modelo demanda-controle de Karasek, versão sueca de Theorell)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Universidade de Brasília, tese de doutorado (orient. Ana Magnólia Mendes)</t>
+          <t>Revista de Saúde Pública (USP), v. 38, n. 2, p. 164-171</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>repositorio.unb.br/bitstream/10482/15420/1/2013_EmilioPeresFacas.pdf</t>
+          <t>scielo.br/j/rsp/a/55vCVJNvKpJcsGNjhpq5W4r</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>2013 (4 escalas)</t>
+          <t>2004 (17 itens)</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Ano da tese que validou o protocolo.</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Vigente (conferir)</t>
+          <t>Ano da adaptação e validação para o português.</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Vigente</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Sim: instrumento brasileiro, validado na própria tese.</t>
+          <t>Sim: o próprio artigo (reprodutibilidade 0,88 demanda; 0,87 controle; 0,85 apoio social).</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Acesso aberto; citar a fonte.</t>
+          <t>Artigo de acesso aberto; itens no anexo. O JCQ original de Karasek (versão longa) é licenciado e não foi usado.</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>FACAS, E. P. Protocolo de Avaliação dos Riscos Psicossociais no Trabalho: contribuições da psicodinâmica do trabalho. 2013. Tese (Doutorado) - Universidade de Brasília, Brasília, 2013.</t>
+          <t>ALVES, M. G. M. et al. Versão resumida da "job stress scale": adaptação para o português. Revista de Saúde Pública, São Paulo, v. 38, n. 2, p. 164-171, 2004.</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>Protocolo completo no Anexo 5 (p. 185 a 191). Há livro do autor de 2021 (DOI 10.22350/9786559173686); não foi possível confirmar se mudou algum item.</t>
+          <t>Continua sendo a versão de referência no Brasil. DOI 10.1590/S0034-89102004000200003.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
+          <t>2. Questionarios validados no Brasil/PROART - tese UnB Facas 2013 (protocolo no Anexo 5).pdf</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Protocolo de Avaliação dos Riscos Psicossociais no Trabalho (PROART)</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Universidade de Brasília, tese de doutorado (orient. Ana Magnólia Mendes)</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>repositorio.unb.br/bitstream/10482/15420/1/2013_EmilioPeresFacas.pdf</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>2013 (4 escalas)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Ano da tese que validou o protocolo.</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Vigente (conferir)</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Sim: instrumento brasileiro, validado na própria tese.</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Acesso aberto; citar a fonte.</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>FACAS, E. P. Protocolo de Avaliação dos Riscos Psicossociais no Trabalho: contribuições da psicodinâmica do trabalho. 2013. Tese (Doutorado) - Universidade de Brasília, Brasília, 2013.</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Protocolo completo no Anexo 5 (p. 185 a 191). Há livro do autor de 2021 (DOI 10.22350/9786559173686); não foi possível confirmar se mudou algum item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
           <t>(a baixar) Chor et al 2008</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Validação brasileira do ERI</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Cadernos de Saúde Pública, v. 24, n. 1, p. 219-224</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>scielo.br/j/csp/a/DHm6M7KNMMXbJkxMtgZMDYs</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>2008</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>Ano da validação.</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Vigente</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr"/>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr"/>
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Acesso aberto.</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr"/>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr"/>
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>SciELO fora do ar no download (erro 503); baixar depois. DOI 10.1590/S0102-311X2008000100022.</t>
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2. Questionarios validados no Brasil/HSE Indicator Tool - questionario 35 itens (Reino Unido).pdf</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>HSE Management Standards Indicator Tool (35 itens)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Health and Safety Executive (governo do Reino Unido)</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>hse.gov.uk/stress/assets/docs/indicatortool.pdf</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Versão oficial distribuída hoje no site do HSE.</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Não: sem validação brasileira localizada. Referência internacional complementar (o Manual do GRO admite instituição de SST internacional).</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Material público do governo britânico; citar a fonte.</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>HEALTH AND SAFETY EXECUTIVE. HSE Management Standards Indicator Tool. Reino Unido: HSE, 2004.</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Seis fatores: demandas, controle, suporte (chefia e colegas), relacionamentos, papel e mudanças. Formulário também em 3. Questionarios oficiais usados como base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>2. Questionarios validados no Brasil/HSE Indicator Tool - manual (Reino Unido).pdf</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Manual do usuário do Indicator Tool</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Idem</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>hse.gov.uk/stress/assets/docs/indicatortoolmanual.pdf</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Idem.</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Idem.</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Idem.</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr"/>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Como aplicar e apurar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>2. Questionarios validados no Brasil/HSE Analysis Tool - planilha de apuracao (Reino Unido).xls</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Analysis Tool (planilha oficial de apuração)</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Idem</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>hse.gov.uk/stress/assets/docs/analysistool.xls</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Última gravação do arquivo oficial.</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Idem.</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Idem.</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr"/>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Planilha Excel do HSE que calcula os resultados por fator.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:K15"/>
+  <autoFilter ref="A3:K19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5156,7 +5569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5480,8 +5893,30 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>3. Referência internacional complementar</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>HSE Management Standards Indicator Tool (Health and Safety Executive, Reino Unido, 2004)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Ferramenta de instituição de SST internacional</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Seis fatores de estresse. Sem validação brasileira localizada; reforça itens de demandas, controle, suporte, relacionamentos, papel e mudanças.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:D16"/>
+  <autoFilter ref="A3:D17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>